<commit_message>
feat(front): e-mail na validação, motivo dos ajustes e linha do código repetido
- Coluna opcional email: padronizada (espaços e minúsculas) e conferida;
  formato errado vira o erro "E-mail inválido".
- Código repetido informa em que linha o código apareceu primeiro.
- Ajustes automáticos ganham motivo (Espaços extras, Maiúsculas e
  minúsculas, Escrita padronizada, Formato do valor), com o getter
  padronizacoesPorMotivo e a coluna Motivo no relatório.
- Planilhas de modelo e de teste geradas de novo com a coluna email.
- Relatório da atividade "Pinia - Validação de Planilha" em docs/.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/frontend-vue/public/modelo-clientes.xlsx
+++ b/frontend-vue/public/modelo-clientes.xlsx
@@ -400,7 +400,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J3"/>
+  <dimension ref="A1:K3"/>
   <cols>
     <col min="1" max="1" width="18.83203125" customWidth="1"/>
     <col min="2" max="2" width="18.83203125" customWidth="1"/>
@@ -412,6 +412,7 @@
     <col min="8" max="8" width="20.83203125" customWidth="1"/>
     <col min="9" max="9" width="18.83203125" customWidth="1"/>
     <col min="10" max="10" width="18.83203125" customWidth="1"/>
+    <col min="11" max="11" width="18.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -445,6 +446,9 @@
       <c r="J1" t="str">
         <v>uf</v>
       </c>
+      <c r="K1" t="str">
+        <v>email</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
@@ -477,6 +481,9 @@
       <c r="J2" t="str">
         <v>SP</v>
       </c>
+      <c r="K2" t="str">
+        <v>financeiro@metalurgicahorizonte.com.br</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
@@ -509,17 +516,20 @@
       <c r="J3" t="str">
         <v>SP</v>
       </c>
+      <c r="K3" t="str">
+        <v>compras@comercialvitoria.com.br</v>
+      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:J3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:K3"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F16"/>
+  <dimension ref="A1:F17"/>
   <cols>
     <col min="1" max="1" width="22.83203125" customWidth="1"/>
     <col min="2" max="2" width="22.83203125" customWidth="1"/>
@@ -749,29 +759,49 @@
         <v>Opcional; se preenchida, 2 letras (sp vira SP)</v>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" t="str">
-        <v>Como usar</v>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>email</v>
+      </c>
+      <c r="B12" t="str">
+        <v>E-mail</v>
+      </c>
+      <c r="C12" t="str">
+        <v>texto</v>
+      </c>
+      <c r="D12" t="str">
+        <v>Não</v>
+      </c>
+      <c r="E12" t="str">
+        <v>contato@empresa.com.br</v>
+      </c>
+      <c r="F12" t="str">
+        <v>Opcional; se preenchido, formato nome@empresa.com.br (maiúsculas e espaços são corrigidos)</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>Preencha a aba "upload_clientes" a partir da linha 2, sem mudar os nomes das colunas.</v>
+        <v>Como usar</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>Formatos aceitos: .xlsx, .xls, .csv. Limite: 5 MB e 20.000 linhas.</v>
+        <v>Preencha a aba "upload_clientes" a partir da linha 2, sem mudar os nomes das colunas.</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
+        <v>Formatos aceitos: .xlsx, .xls, .csv. Limite: 5 MB e 20.000 linhas.</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
         <v>Use apenas dados fictícios ou autorizados.</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F16"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F17"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>